<commit_message>
docs: add Roadmap sheet to OBSERVATIONS_UI.xlsx
R1-R5 produit (Stripe, limites Free, email confirm, domaine, test Barbara)
R6-R10 qualite tech (E2E, TypeScript strict, ARIA, Performance, Sentry)
R11-R14 phase 2 (React Native, gamification, push, calendrier)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/OBSERVATIONS_UI.xlsx
+++ b/docs/OBSERVATIONS_UI.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Observations UI" sheetId="1" r:id="rId1"/>
+    <sheet name="Roadmap" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -398,14 +399,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F22"/>
-  <cols>
-    <col min="1" max="1" width="4.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="52.83203125" customWidth="1"/>
-    <col min="4" max="4" width="52.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -852,4 +845,323 @@
     <ignoredError numberStoredAsText="1" sqref="A1:F22"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F15"/>
+  <cols>
+    <col min="1" max="1" width="5.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="4" width="65.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>N</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Categorie</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Titre</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Priorite</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Statut</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>R1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Stripe / paiement</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Integrer Stripe Checkout pour upgrade Free vers Premium. Webhook pour activer le flag premium en DB.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Critique</v>
+      </c>
+      <c r="F2" t="str">
+        <v>A faire</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>R2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Limites Free enforced</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Max 2 membres + quota IA (5 generations/mois) bloques cote serveur avec message upgrade.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Critique</v>
+      </c>
+      <c r="F3" t="str">
+        <v>A faire</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>R3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Email confirmation</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Reactiver la confirmation email dans Supabase Auth pour valider les comptes.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="F4" t="str">
+        <v>A faire</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>R4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Nom de domaine</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Trouver alternative a yova.app (pris). Tester yova.fr, getyova.com, yova.co.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="F5" t="str">
+        <v>A faire</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>R5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Produit</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Test Barbara</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Parcours complet : onboarding, creation tache, validation, analytics.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="F6" t="str">
+        <v>A faire</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>R6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Qualite tech</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Tests E2E</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Cypress ou Playwright : couvrir onboarding, creation tache, completion, planning.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="F7" t="str">
+        <v>A faire</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>R7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Qualite tech</v>
+      </c>
+      <c r="C8" t="str">
+        <v>TypeScript strict</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Activer strict:true dans tsconfig + corriger les 22+ casts incorrects.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Moyenne</v>
+      </c>
+      <c r="F8" t="str">
+        <v>A faire</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>R8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Qualite tech</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Accessibilite ARIA</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Ajouter aria-label sur boutons icones, roles sur modals, navigation clavier.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Moyenne</v>
+      </c>
+      <c r="F9" t="str">
+        <v>A faire</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>R9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Qualite tech</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Performance</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Lazy loading images, code splitting, optimiser LCP / TTI. Audit Lighthouse &gt; 90.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Moyenne</v>
+      </c>
+      <c r="F10" t="str">
+        <v>A faire</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>R10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Qualite tech</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Monitoring Sentry</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Integrer Sentry pour capturer les erreurs runtime + alertes en prod.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="F11" t="str">
+        <v>A faire</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>R11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Phase 2</v>
+      </c>
+      <c r="C12" t="str">
+        <v>React Native / PWA</v>
+      </c>
+      <c r="D12" t="str">
+        <v>App mobile native (Expo) ou PWA installable avec push notifications.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Future</v>
+      </c>
+      <c r="F12" t="str">
+        <v>A planifier</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>R12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Phase 2</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Gamification</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Points, streaks, mascotte qui evolue selon activite du foyer.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Future</v>
+      </c>
+      <c r="F13" t="str">
+        <v>A planifier</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>R13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Phase 2</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Notifications push</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Rappels taches dues, felicitations, relances intelligentes via IA.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Future</v>
+      </c>
+      <c r="F14" t="str">
+        <v>A planifier</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>R14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Phase 2</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Integration calendrier</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Sync Google Calendar / Apple Calendar pour les taches planifiees.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Future</v>
+      </c>
+      <c r="F15" t="str">
+        <v>A planifier</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>